<commit_message>
remove scoring answer leaks and strengthen Windows audit
</commit_message>
<xml_diff>
--- a/artifacts/任务规格转化.xlsx
+++ b/artifacts/任务规格转化.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格转化" sheetId="1" r:id="Rb77d573f54374cff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格转化" sheetId="1" r:id="R688b2e2e9fb945fd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -447,18 +447,18 @@
     </x:row>
     <x:row r="18" ht="33" customHeight="1">
       <x:c r="A18" s="5" t="str">
-        <x:v>可验证点</x:v>
+        <x:v>结果核对</x:v>
       </x:c>
       <x:c r="B18" s="5" t="str">
-        <x:v>物理行去向、压制原因、URL字段、策略指纹、源码坐标、严重级别、最长前缀与报告排序</x:v>
+        <x:v>物理行去向、压制原因、URL字段、策略指纹、源码坐标、严重级别、最长前缀与报告排序均可从输入复算</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="33" customHeight="1">
       <x:c r="A19" s="5" t="str">
-        <x:v>不适合作为评分点的内容</x:v>
+        <x:v>实现自由度</x:v>
       </x:c>
       <x:c r="B19" s="5" t="str">
-        <x:v>函数拆分、变量名、注释、内部索引结构、CSV必要引号和LF或CRLF行尾</x:v>
+        <x:v>函数拆分、变量名、注释和内部索引结构可以不同，CSV允许必要引号及LF或CRLF行尾</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>